<commit_message>
Deepen KB to 500-900 chars/unit, add ashnav_ref, shift sources to Yad Vashem/ORT, merge duplicates
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/history_agent/source1_marking_schemes.xlsx
+++ b/data/history_agent/source1_marking_schemes.xlsx
@@ -4065,17 +4065,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ערים וקהילות › העיר המוסלמית › צמיחת הערים ובגדד</t>
+          <t>ערים וקהילות › העיר המוסלמית › צמיחת הערים ובגדאד</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>ייסוד בגדד ושיקוליו; בגדד כמרכז סחר; המבנה החברתי בעיר</t>
+          <t>ייסוד בגדאד ושיקוליו; בגדאד כמרכז סחר; המבנה החברתי בעיר</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>ח'ליפות עבאסית, בגדד, רבעים, מרכז סחר, מבנה חברתי</t>
+          <t>ח'ליפות עבאסית, בגדאד, רבעים, מרכז סחר, מבנה חברתי</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">

</xml_diff>